<commit_message>
update cholesterol titles 656fa94b43378a075b8e9b8c1b67c2d1eec30e34
</commit_message>
<xml_diff>
--- a/nr-add-lipids/ig/StructureDefinition-mesures-observation-cholesterol-hdl.xlsx
+++ b/nr-add-lipids/ig/StructureDefinition-mesures-observation-cholesterol-hdl.xlsx
@@ -45,7 +45,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Cholestérol HDL</t>
+    <t>Cholestérol - HDL</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-27T15:45:03+00:00</t>
+    <t>2025-03-27T15:47:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>